<commit_message>
Jon Excel updated notes
</commit_message>
<xml_diff>
--- a/documentation/Jons_Cidy_Intent_Test_Cases_90.xlsx
+++ b/documentation/Jons_Cidy_Intent_Test_Cases_90.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RRAPOPOR\Documents\Cidy testing\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/831750913a0e3f96/UN/Cidy/cidy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B301336-FE44-41E3-9BB8-269871358495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{2B301336-FE44-41E3-9BB8-269871358495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4A99D31-13C8-4E3D-A93A-A374A720AB53}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34464" yWindow="0" windowWidth="15960" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="358">
   <si>
     <t>Scenario</t>
   </si>
@@ -608,34 +608,6 @@
     <t>Test Date</t>
   </si>
   <si>
-    <t>Answer: Intent Identified: You are seeking a comprehensive summary of the required sections and planning/design requirements for a Development Account (DA) concept note, referencing the latest (19th tranche) guidelines, templates, and review checklists, with a focus on project planning, objectives, budget, results framework, quality assurance, internal review, submission, and implementing entity.
-Required Sections for a DA Concept Note (19th Tranche):
-Background: Describe the issue, context, human rights, gender, disability inclusion, demand from Member States, tentative target countries, and link to implementing entity.
-Fascicle Note: Title, implementing entity and partners, SDG targets, objective, project plan for 2027–2030, budget summary, and additional required tables.
-Outcomes and Outputs (Results Framework): At least two outcomes and linked outputs with strong logical linkages.
-UN System Coordination: Plans for engaging RCOs and UN Country Teams, and key partnerships.
-Budget Narrative: Detailed breakdown by budget class using required tables and formats.
-Planning/Design Requirements:
-Use the latest template (Annex 1).
-Quality Assurance and Internal Review: Internal quality review using the provided checklist.
-Submission Requirements: Submit twice the number of projects as funded previously, prioritize special needs countries, and meet criteria for joint projects.
-Implementing Entity: Must be one of the 10 DA entities, clearly stating lead, joint, and collaborating entities.
-Key Quality and Planning Considerations:
-Link to tranche theme and capacity development.
-Address implementing unit capacity.
-Exclude evaluation costs at concept note stage.
-Provide all data in requested format.
-Reference to Latest Guidelines, Templates, and Checklists:
-Guidelines: 19th tranche Concept Note Guidelines.
-Template: 19th tranche Concept Note Template (Annex 1).
-Review Checklist: 19th tranche Concept Note Review Checklist for DA Focal Points.
-Sources:
-T19 Concept Note Guidelines.docx
-T19 Concept Note Template.docx
-T19 Concept Note Review Checklist for DA Focal Points.docx
-Confidence: Very High</t>
-  </si>
-  <si>
     <t>FoundAnswer</t>
   </si>
   <si>
@@ -648,66 +620,7 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Answer: You are seeking a comprehensive, step-by-step overview of the process and requirements for preparing a Development Account (DA) project document for the latest tranche, including all key elements, required tools, and quality assurance steps.
-Use the Most Recent Guidance and Templates
-Always use the latest tranche’s guidelines and templates (currently the 19th tranche, T19) for project documents, unless an earlier tranche is specifically requested.
-The main sources are the T19 Project Document Guidelines, the T19 Project Document Template, the T19 Project Document Annex (Excel), and the T19 Project Document Review Checklist for DA Focal Points.
-The guidelines provide detailed instructions for each section; the template is for drafting; the Excel annex is for workplans and budget tables; the checklist is for internal review before submission.
-Project Planning and Preparation Steps
-Expand the concept note into a full project document, using feedback from the concept note review.
-Drafting typically occurs from May to September of the relevant year (e.g., 2026 for T19).
-Confirm target countries and consult the Resident Coordinator Office (RCO) in each target country during drafting.
-For joint projects, ensure all jointly implementing entities agree on strategy, roles, and budget distribution before submission.
-Structure and Key Elements of the Project Document
-Executive Summary: Project code/title, implementing entity, jointly implementing/collaborating entities, implementing partners, end date, budget, use of IPMR, target countries, SDG relevance, and a brief description (max 300 words).
-Demand, Context, and Analysis: Selection and rationale for target countries, context and situation analysis (including gender/disability/vulnerable groups), country-level analysis, and (optionally) stakeholder analysis.
-Project Strategy:
-Envisaged change in the countries (concrete change sought).
-Theory of change narrative and main assumptions.
-Results framework (objective, outcomes, indicators, baselines, means of verification, outputs).
-Results-based workplan (in Excel annex).
-Risks and mitigating actions.
-Post-project sustainability and scaling-up.
-Lessons learned from past projects.
-Gender Equality and Disability Inclusion: Assign and justify gender and disability markers, ensuring alignment with the results framework.
-Monitoring, Reporting, and Evaluation:
-Explain monitoring arrangements, reporting intervals, and evaluation plans.
-For joint projects over $1 million, include a detailed evaluation plan and annual monitoring calls.
-Mandates, Partnerships, and Coordination Agreements:
-Describe mandates, roles, and responsibilities of all entities.
-For joint projects, confirm shared outcomes and joint outputs, and establish a Project Steering Committee.
-List implementing partners and describe their roles and budget share.
-Document RCO engagement for each target country.
-Budget:
-Complete all required budget tables in the Excel annex, following guidance in section 7 of the guidelines.
-Consult finance colleagues for joint projects.
-Ensure compliance with rules on staff capacity, travel, and use of consultants/partners.
-Quality Assurance and Internal Review
-Use the T19 Project Document Review Checklist for DA Focal Points to ensure all requirements are met before submission.
-The checklist covers all sections, including budget accuracy, alignment of entities, clarity of objectives, results framework, gender/disability markers, monitoring/evaluation, and RCO engagement.
-The DA Focal Point must complete the checklist and confirm internal quality assurance before submission.
-Submission Process
-Submit the draft project document to the DA Programme Management Team (DA-PMT) by the specified deadlines (e.g., 30 June for at least one document per entity, all by 15 September).
-Submissions are accepted on a rolling basis as documents are ready.
-Only submit after thorough internal review and quality control.
-Implementing Entity Requirements
-The lead implementing entity is responsible for overall coordination, quality assurance, and reporting.
-For joint projects, all jointly implementing entities must be involved in design, implementation, monitoring, and evaluation.
-The Project Steering Committee (for joint projects) oversees coordination and performance.
-Summary Table of Required Tools and Elements | Element | Source/Tool | |------------------------------- |----------------------------------------------| | Guidelines | T19 Project Document Guidelines | | Drafting Template | T19 Project Document Template | | Budget/Workplan | T19 Project Document Annex (Excel) | | Quality Assurance | T19 Project Document Review Checklist | | Internal Review | DA Focal Point review and checklist | | Submission | To DA-PMT after internal QA | | Implementing Entity | Lead and (if joint) jointly implementing |
-Sources:
-T19 Project Document Guidelines.docx
-T19 Project Document Template.docx
-T19 Project Document Annex.xlsx
-T19 Project Document Review Checklist for DA Focal Points.docx
-readme.docx
-Confidence: Very High</t>
-  </si>
-  <si>
     <t>Perfomance</t>
-  </si>
-  <si>
-    <t>less than 15secs</t>
   </si>
   <si>
     <t>Answer: I was not able to find information in my knowledge sources that could answer this question.
@@ -718,115 +631,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Answer: Yes, under the Development Account, travel costs are considered eligible expenses. Specifically, the budget class "Travel of Staff (115)" is used exclusively for the travel of UN system-wide staff for all types of travel, including participation in expert groups, workshops, and providing advisory services. However, staff travel costs should not be included under "Grants and Contributions – Workshops/Study Tours (145)", which is reserved for the travel/DSA of participants attending seminars, workshops, study tours, and expert group meetings. The number of staff traveling per activity should be limited, especially if there are consultants traveling for the same activity. For joint projects, careful consideration should be given to the necessity of travel, and hybrid or virtual options should be utilized where possible to manage costs effectively.
-Sources:
-T16 Project Document Guidelines v6 final.pdf
-T19 Concept Note Guidelines.docx
-T18 Project Document Guidelines.docx
-T19 Project Document Guidelines.docx
-Confidence: Very High</t>
-  </si>
-  <si>
-    <t>Answer: 1. Official Guidance and Requirements
-Terminal evaluations are mandatory for all DA projects with a budget of USD 1 million or more and are strongly encouraged for others selected at midterm.
-The process and structure are governed by the DA Project Evaluation Guidelines, the Administrative Instructions on Evaluation in the UN Secretariat (ST/AI/2021/3), and tranche-specific guidance notes. For joint projects, refer to the DA guidance note on terminal evaluation of joint projects (latest version: June 2023, V.1).
-Evaluation Design Steps
-Preparatory Phase
-Develop a detailed tentative evaluation plan as part of the project document, including:
-Timeline (evaluation report due within 9 months of project completion for projects ≥ USD 1 million; 6 months for others)
-Target users and intended use of results
-Management and support arrangements
-Preliminary methodology
-Tentative budget (up to 4% of final project budget)
-Follow-up plan
-Development of Terms of Reference (TOR)
-Start at least 6 months before project completion.
-TOR should include:
-Purpose and objectives of the evaluation
-Project context and description
-Evaluation scope, criteria, and tentative questions
-Methodology (see below)
-List of key stakeholders
-Organization, roles, responsibilities, workplan, and deliverables
-Dissemination strategy
-Evaluation budget and required evaluator qualifications
-Integration of human rights, gender equality, and, where possible, disability perspectives
-Required Methodology
-Use a mixed-methods approach, ensuring triangulation of data sources for confidence in findings.
-Typical methods include:
-Desk review of project documents and data
-Interviews (in-person or remote)
-Focus group discussions
-Online surveys
-Field visits (for beneficiary feedback not easily collected remotely)
-Observation of workshops/meetings
-Methodology should be tailored to the project’s scope, activities, geographic coverage, and available data and budget.
-For joint projects, ensure data collection covers all implementing entities, not just the lead.
-Evaluation Report Structure
-Use the DA project evaluation report template (or, if required, the entity’s own template with all DA-required elements included).
-Key sections:
-Executive summary
-Description of the project (context, objectives, strategies, partners, resources, SDG links, innovative elements)
-Evaluation objectives, scope, and questions
-Methodology (including rationale, data sources, sampling, ethical standards, integration of gender/human rights/disability)
-Findings (evidence-based, linked to criteria/questions, gender-disaggregated where relevant)
-Conclusions
-Recommendations (practical, feasible, directed to intended users)
-Lessons learned and good practices (for broader dissemination)
-Annexes (TOR, results framework, evaluation matrix, data collection tools, list of interviews/documents)
-Management and Follow-up
-Each implementing entity is responsible for developing a management response to recommendations within 3 months of report finalization.
-Management responses and evaluation reports are published on the DA website and entities’ own sites.
-Entities must track implementation of accepted recommendations.
-Reference to Official Guidance
-Use the latest DA Project Evaluation Guidelines, tranche-specific guidance notes, and the DA guidance note on terminal evaluation of joint projects (June 2023, V.1) for detailed instructions and templates.
-Sources:
-DA guidance note on terminal evaluation of joint projects v1.pdf
-Guide to the Development Account 2025.pdf
-T15 DA project evaluation report template (annotated).docx
-T15 DA guidance note on project evaluations - re re final 2.3.2026.docx
-Confidence: Very High</t>
-  </si>
-  <si>
-    <t>Answer: To initiate a new Development Account (DA) project, follow these steps:
-Understand the Planning Cycle: The DA project cycle begins about 1.5 years before the four-year implementation period. Each tranche is guided by a theme selected by the DA Steering Committee and approved by the Programme Manager.
-Draft a Concept Note: This is the first required document. It should align with the tranche theme, demonstrate demand from target countries, and outline objectives, expected results, and partnerships. Use the latest concept note guidelines and template from the DA website and SharePoint. Internal quality review by the DA Focal Point is mandatory before submission, typically due mid-November of the planning year.
-Shortlisting and Approval: Concept notes are reviewed by the DA-PMT, shortlisted, and approved by the DA Steering Committee and Programme Manager. Shortlisted projects are included in the UN Programme Budget for General Assembly approval.
-Draft a Project Document: After shortlisting, develop a detailed project document including theory of change, results framework, monitoring plan, and budget. Use tranche-specific guidelines and templates. Internal quality assurance and consultations with Resident Coordinator Offices are required. Deadline is typically mid-September of the planning year.
-Review and Finalization: The DA-PMT reviews and provides feedback. After revisions and final approval, the project is ready for fund allocation following General Assembly approval.
-Required Initial Documents:
-Concept Note (latest guidelines and template)
-Project Document (latest guidelines and template, after shortlisting)
-Always use the most recent tranche guidelines and coordinate with your DA Focal Point throughout the process.
-Sources:
-Guide to the Development Account 2025.pdf
-T19 Concept Note Guidelines.docx
-T19 Project Document Guidelines.docx
-Confidence: Very High</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Answer: When starting a new Development Account (DA) project, you should always use the guidance for the most recent tranche available. The DA knowledge base specifies that the files and guidelines are organized by tranche number (e.g., T14, T15, T16, etc.), and you should reference the highest-numbered (most recent) tranche for the most up-to-date instructions. Only refer to earlier tranche guidance if you are specifically asked about a previous tranche. This ensures your project planning and documentation align with the latest requirements and processes set by the DA.
-Sources:
-readme.docx
-Confidence: Very High
- </t>
-  </si>
-  <si>
-    <t>Answer: Yes, there is a checklist available for reviewing Development Account (DA) concept notes. The checklist is designed to assist DA Focal Points in reviewing each concept note before submission. It covers key sections such as:
-General: Ensuring the correct template is used and that the implementing section has sufficient resources.
-Background: Explanation of the issue, context, target countries, demand, and connection to the implementing entity’s work.
-Fascicle Note: Format, objective, project plan, and word count.
-Additional Data: Completion and formatting of required tables.
-Outcomes and Outputs: Sufficiency and clarity of outputs and their link to outcomes.
-UN System: Specific plans for engaging Resident Coordinator Offices (RCOs) and explanation of partnerships.
-Budget Summary: Correct format and accuracy of figures.
-The checklist is intended to ensure internal quality review and adherence to guidelines before submission to the DA Team. It is referenced in the most recent tranche guidance and is available as an annex to the concept note guidelines for the 19th tranche.
-Sources:
-T19 Concept Note Review Checklist for DA Focal Points.docx
-T19 Concept Note Guidelines.docx
-Confidence: Very High</t>
-  </si>
-  <si>
     <t>CorrectSources</t>
   </si>
   <si>
@@ -834,9 +638,6 @@
   </si>
   <si>
     <t>General Notes</t>
-  </si>
-  <si>
-    <t>Answer appears twice.</t>
   </si>
   <si>
     <t>I am sorry, I was not able to find a confident answer to your question in my knowledge sources. I am still under development and new knowledge is coming in every week. See ​Cidy Knowledge Status​ for more information.
@@ -1148,318 +949,732 @@
 </t>
   </si>
   <si>
-    <t>Answer: The responsibility for maintaining Cidy's knowledge base and ensuring its information is up to date lies with the Knowledge Control Center. This component tracks knowledge folders, source-use instructions, manager updates, route coverage, and YAML work needed to keep response topics aligned. The governance and maintenance architecture also includes an inventory generator, refresh workflow, and structural test runner to support ongoing updates and quality control. Human-in-the-loop processes are in place for unresolved or low-confidence cases, which are routed to feedback or escalation rather than being treated as definitive answers. This ensures that the knowledge base remains current and reliable as the system matures and new materials are added or updated.
+    <t>Did get asked multiple choice; DEBUG - Pass 2 result: Broad DA source (Pass 1 was blank)
+Query sent:
+Response:</t>
+  </si>
+  <si>
+    <t>Claude Found?</t>
+  </si>
+  <si>
+    <t>Happy path - DA project planning [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA project document [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA monitoring and reporting [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA budget eligibility [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA Section 35 signal [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA evaluation design [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA evaluation template [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA general start [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA latest tranche [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - DA checklist [DA]</t>
+  </si>
+  <si>
+    <t>Happy path - project evaluation evidence [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - evaluation recommendations [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - lessons learned [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - recurring evaluation findings [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - evaluation weaknesses [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - partnerships in evaluations [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - sustainability recommendations [Evaluation]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development CD Strategy [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development Steering Committee [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development TAG [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development general [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development annual progress report template [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development final report template [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development project document preparation [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development implementing partner agreement [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development grants due diligence [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development IPGC templates [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC budget and finance [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC governance [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC roles [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC programme design standards [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC evaluation criteria [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC reports [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - PDF / UNPDF [PDF]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy coverage [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy maintenance [About Cidy]</t>
+  </si>
+  <si>
+    <t>Clarification path - fund to DA [DA]</t>
+  </si>
+  <si>
+    <t>Clarification path - fund to RPTC [RPTC]</t>
+  </si>
+  <si>
+    <t>Clarification path - fund to PDF [PDF]</t>
+  </si>
+  <si>
+    <t>Clarification path - fund not sure [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain to DA [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain to Programme Development [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain to Evaluation Evidence [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain to About Cidy [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain to RPTC [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain typed DA [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain typed Development Account [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - domain typed UNPDF [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - artifact concept note [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - artifact evaluation report [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - artifact progress report [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - artifact management response [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - second attempt succeeds [Not Sure]</t>
+  </si>
+  <si>
+    <t>Clarification path - max attempts dead end [Not Sure]</t>
+  </si>
+  <si>
+    <t>Vague path - domain clarification [Not Sure]</t>
+  </si>
+  <si>
+    <t>Vague path - template clarification [Not Sure]</t>
+  </si>
+  <si>
+    <t>Vague path - report clarification [Not Sure]</t>
+  </si>
+  <si>
+    <t>Vague path - guidance clarification [Not Sure]</t>
+  </si>
+  <si>
+    <t>Vague path - project support clarification [Not Sure]</t>
+  </si>
+  <si>
+    <t>Out of scope - weather [OOS]</t>
+  </si>
+  <si>
+    <t>Out of scope - sports [OOS]</t>
+  </si>
+  <si>
+    <t>Out of scope - poem [OOS]</t>
+  </si>
+  <si>
+    <t>Out of scope - laptop help [OOS]</t>
+  </si>
+  <si>
+    <t>Out of scope - stock investment [OOS]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC activity proposal template [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC common reporting standards [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC IRA guidance [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC activity report template [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC planning and approval process [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC 2024 achievements [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC 2024 countries requests interventions [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC implementing entities [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC SIDS LDC LLDC support [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - RPTC future recommendations [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development Resident Coordinator mission notice [RPTC]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development UNSDCF alignment [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development UNCT membership [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development strategic priorities [PD]</t>
+  </si>
+  <si>
+    <t>Happy path - Programme Development service delivery model [PD]</t>
+  </si>
+  <si>
+    <t>Clarification path - Programme Development strategy from broad Cidy question [Not Sure]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy overview [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy comparison [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy user questions [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy prompt examples [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy routing flow [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy low confidence  [About Cidy]</t>
+  </si>
+  <si>
+    <t>Happy path - About Cidy architecture  [About Cidy]</t>
+  </si>
+  <si>
+    <t>Greeting path - English greeting only [Greeting]</t>
+  </si>
+  <si>
+    <t>Greeting path - Multilingual greeting only  [Greeting]</t>
+  </si>
+  <si>
+    <t>Greeting guard - greeting plus substantive question [Greeting]</t>
+  </si>
+  <si>
+    <t>Exit Cidy flow command - exact phrase [Exit Flow]</t>
+  </si>
+  <si>
+    <t>Exit Cidy flow command - Cindy typo [Exit Flow]</t>
+  </si>
+  <si>
+    <t>Return to Cidy rescue path  [Exit Flow]</t>
+  </si>
+  <si>
+    <t>Happy path - Country Data active projects by country [Country Data]</t>
+  </si>
+  <si>
+    <t>Regression - broad country work routes to Country Data [Country Data]</t>
+  </si>
+  <si>
+    <t>Happy path - Country Data proposal year list [Country Data]</t>
+  </si>
+  <si>
+    <t>Happy path - Country Data LDC activity count [Country Data]</t>
+  </si>
+  <si>
+    <t>Topic Area</t>
+  </si>
+  <si>
+    <t>Answer appears twice. Investigating -- sources are identical which is good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+Answer: A DA concept note for the 19th tranche must include the following main elements and adhere to specific formatting and content requirements:
+Background
+Description of the issue the project intends to address, including broader context.
+Reference to a human rights-based approach, ‘leaving no one behind’, gender considerations, and disability inclusion.
+Specific demand/requests from Member States for the proposed support.
+Tentative list of potential target countries, if known.
+Connection to the work of the implementing entity/entities and their comparative advantages.
+Fascicle Note (to be used in the Supplementary Information of the Proposed Programme Budget)
+a. Title: Compelling, positive, concise, and includes thematic area and geographical scope.
+b. Implementing entities and partners: List all 10 DA implementing entities involved, starting with the lead, then joint, then collaborating entities, using the required format.
+c. Relationship to the SDG targets: List up to 10 essential SDG targets in ascending order (numbers only).
+d. Objective: One-sentence intended goal, referencing beneficiaries, geographical scope, and substantive focus. Avoid process descriptions or internal UN work verbs.
+e. Project plan for 2027-2030.
+f. Budget summary.
+Additional Data Needed for the Fascicle
+Data for analysis of the tranche and proposed projects, in the requested format.
+Outcomes and Outputs
+Outputs must be sufficient to achieve outcomes, and outcomes must contribute to the objective.
+Outputs should describe specific actions, products, or reports in enough detail for external understanding.
+UN System Coordination
+Plans for engaging Resident Coordinator Offices (RCOs) and partnerships with other UN entities, funds, programmes, and country teams.
+Budget Narrative
+Figures must be in the required format (one decimal place, in thousands of USD).
+All budget categories must sum to the total.
+Additional Requirements
+Use the separate template provided (Annex 1) for drafting.
+The fascicle note should be no longer than one page.
+All sections must follow the format and guidelines strictly, as these are used for official budget presentations.
+A review checklist (Annex 2) is available for internal quality assurance before submission.
+These requirements are based on the most recent (19th tranche) guidelines available. For drafting, always use the latest template and ensure all sections are complete and in the correct format.
+Sources:
+​T19 Concept Note Guidelines.docx​
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+Confidence: High
+</t>
+  </si>
+  <si>
+    <t>timer broken, investigating</t>
+  </si>
+  <si>
+    <t>Answer appears twice, took multiple attempts.</t>
+  </si>
+  <si>
+    <t>Yes*</t>
+  </si>
+  <si>
+    <t>Answer: To prepare a project document for the Development Account (DA), follow these steps, referencing the most recent (19th tranche) guidance:
+Use the Latest Guidelines and Templates
+Always use the most recent tranche’s guidelines and templates (e.g., T19 for the 19th tranche) for project document preparation.
+The “T19 Project Document Guidelines” provide detailed instructions for each section, and the “T19 Project Document Template” is used for drafting. There is also a separate Excel file (“T19 Project Document Annex”) for workplans and budget annexes.
+Drafting the Project Document
+Expand on the approved concept note, incorporating any feedback received.
+Complete all required sections in the template, including:
+Executive Summary (project code, title, implementing entities, partners, budget, target countries, SDGs, brief description)
+Demand, Context, and Analysis (selection of target countries, context, country-level analysis, stakeholder analysis)
+Project Strategy (define the envisaged change, theory of change narrative, results framework)
+Gender Equality and Disability Inclusion
+Monitoring, Reporting, and Evaluation
+Mandates, Partnerships, and Coordination Agreements
+Budget (using the Excel annex).
+Key Requirements and Steps
+Engage with monitoring and evaluation colleagues to develop the results framework and define achievement indicators.
+For projects with a budget of $1 million or more, include an evaluation plan and involve relevant officers in preparation.
+Conduct an entity-level quality assurance review, using the standard checklist, and consult with implementing partners and the Resident Coordinator’s Office (RCO) in each target country.
+Submit the draft project document to the DA-PMT for review and revision, responding to comments as needed.
+Once finalized and aligned with guidelines, the project document is eligible for fund allocation after GA approval.
+Where to Find Resources
+The latest guidelines, templates, and checklists are available on the DA SharePoint Site and DA website.
+Only reference templates directly if the question is about their structure; otherwise, rely on the guidelines for content and process.
+Sources:
+​Guide to the Development Account 2025.pdf​
+​T19 Project Document Guidelines.docx​
+​T19 Project Document Template.docx​
+​readme.docx​
+Confidence: Very High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer: Yes, under the Development Account, travel costs are considered eligible expenses. The budget class "Travel of Staff (115)" is specifically designated for the travel of UN system-wide staff, covering transportation costs incurred by staff members to carry out missions in support of the implementation of their mandates. This includes participation in expert groups, workshops, and providing advisory services. However, staff travel costs should not be included under "Grants and Contributions – Workshops/Study Tours (145)", and the number of staff traveling per activity should be limited, especially if consultants are also traveling for the same activity. Additionally, travel costs for consultants may be included under the "Consultants (105)" budget class, as part of their fees if relevant. It is also noted that high travel expenses are scrutinized, so travel costs should be weighed carefully and hybrid or virtual options should be considered where possible.
+Sources:
+​T19 Project Document Guidelines.docx​
+​T18 Project Document Guidelines.docx​
+​T16 Project Document Guidelines v6 final.pdf​
+Confidence: High
+</t>
+  </si>
+  <si>
+    <t>Answer displays twice</t>
+  </si>
+  <si>
+    <t>Answer: Section 3.5 of the Development Account (DA) guidelines addresses "Project Governance and Coordination Arrangements" in project design. It emphasizes the need to:
+Clearly define project governance arrangements, including roles, responsibilities, hierarchy, and communication lines, often illustrated with a diagram.
+Link team member responsibilities to project outcomes and outputs.
+For projects with multiple implementing entities, consider centralized management and funding led by a designated lead entity to improve efficiency and coherence.
+Make lines of accountability explicit in the governance diagram.
+Provide a detailed list of UN partner entities and implementation partners, clarifying that beneficiaries are not considered implementation partners.
+Describe how different actors will collaborate to achieve project objectives and impact.
+Ensure the project document is shared with all implementing entities and partners, with agreements on roles and responsibilities reached before submission for review.
+Plan early engagement with Resident Coordinator (RC) and UN Country Team (UNCT) in target countries, specifying how RCs/UNCTs will be consulted during design and implementation.
+Reference existing coordination mechanisms and alignment with the UN Sustainable Development Cooperation Framework (UNSDCF).
+These steps are intended to ensure effective management, coordination, and national ownership in project design and implementation.
+Sources:
+​generic_project_document_guidelines_final.docx​
+Confidence: Very High</t>
+  </si>
+  <si>
+    <t>***Answer DOES NOT appear twice (???), follow ups do not yield answers, only new test sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer: Designing a Terminal Evaluation for a DA Project involves several steps:
+Evaluation Terms of Reference (TOR)
+Begin developing the TOR 3–6 months before project completion (at least 6 months for joint projects).
+TOR should include: evaluation purpose, project context and description, evaluation objectives and scope, evaluation criteria and tentative questions, methodology (including data availability), key stakeholders to engage, organization and management arrangements, workplan and deliverables, dissemination strategy, evaluation budget, and required qualifications for evaluators (including experience in gender equality and disability inclusion for relevant projects).
+Methodology
+Use multiple methods and triangulate data for robust findings. Common methods: desk review of project documents, interviews (in-person or remote), focus group discussions, online surveys, field visits (if feasible), observation of project events, and analysis of workshop/meeting recordings.
+Select methods based on data availability, project activities, geographic scope, thematic focus, and budget.
+Evaluation Criteria
+Assess relevance, efficiency, effectiveness, and sustainability.
+Include human rights and gender equality as a separate criterion or within the main criteria.
+Consider adding coherence in line with OECD/DAC standards.
+Report Structure
+Follow the DA evaluation report template, which includes: executive summary (3–4 pages), introduction, project description, evaluation objectives, scope, and questions, methodology, findings, conclusions, recommendations, lessons learned and good practices, and annexes (TOR, results framework, evaluation matrix, data collection tools, interviewee list, document list).
+Official Guidance
+Refer to the DA Evaluation Framework and Project Evaluation Guidelines for detailed requirements.
+For joint projects, consult additional guidance in the DA guidance note on terminal evaluation of joint projects.
+Ensure integration of gender equality, human rights, and disability inclusion throughout the evaluation process.
+Sources:
+​T14 DA guidance note on project evaluations - final 2.27.2025.docx​
+​T15 DA guidance note on project evaluations - re re final 2.3.2026.docx​
+​T14 DA project evaluation report template (annotated).docx​
+​T15 DA project evaluation report template (annotated).docx​
+Confidence: High
+</t>
+  </si>
+  <si>
+    <t>Answer displays twice, answers are identical, but with different formatting? Took multiple attempts to find answer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer: The DA evaluation report template is the standardized format used for reporting on Development Account (DA) project evaluations. The latest version, relevant from the 15th tranche (T15) onward, is the "DA project evaluation report template 02-2026." This template ensures consistency and completeness in evaluation reporting across projects.
+Key Contents of the DA Evaluation Report Template (02-2026):
+Cover Page: Includes project title, evaluation period, evaluator(s), evaluation manager(s), and implementing entity’s logo.
+Table of Contents: Lists all sections and annexes.
+List of Acronyms and Abbreviations
+Executive Summary: A stand-alone section (3-4 pages) summarizing the project, evaluation purpose, objectives, scope, methodology, key findings, conclusions, and recommendations.
+Introduction
+Description of the Project:
+Background
+Project objectives and expected results
+Project strategies and key activities
+Beneficiaries and target countries
+Key partners and stakeholders
+Resources
+Link to the Sustainable Development Goals (SDGs)
+Innovative elements (if applicable)
+Evaluation Objectives, Scope, and Questions:
+Purpose and objectives
+Evaluation scope, criteria, and questions
+Methodology
+Findings
+Conclusions
+Recommendations
+Lessons Learned and Good Practices
+Annexes:
+Evaluation Terms of Reference (TORs)
+Project results framework
+Evaluation matrix
+Data collection instruments
+List of individuals interviewed
+List of documents reviewed
+The template is designed to be logical, clear, and complete, supporting both accountability and learning objectives. All DA project evaluation reports are strongly recommended to use this template, or, if an entity uses its own template, to ensure all required DA elements are included either within the main report or as an attachment. The template also supports the dissemination of lessons learned and good practices beyond the implementing entity.
+Sources:
+​T15 DA guidance note on project evaluations - re re final 2.3.2026.docx​
+​DA project evaluation report template 02-2026.docx​
+Confidence: Very High
+</t>
+  </si>
+  <si>
+    <t>Answer DOES not appear twice, first try.</t>
+  </si>
+  <si>
+    <t>debug pass messaging seems to be in wrong sequence.</t>
+  </si>
+  <si>
+    <t>Answer: To ensure you are using the most current and relevant procedures when starting a new Development Account (DA) project, you should follow the guidance document from the highest-numbered tranche available, as this represents the most recent tranche guidance. The files in the Project Planning and Design folder are organized by tranche, with the highest number indicating the latest guidance. Unless you specifically need information from an earlier tranche, always use the most recent tranche guidance to ensure your project aligns with the latest procedures and requirements.
+Sources:
+​readme.docx​
+Confidence: Very High</t>
+  </si>
+  <si>
+    <t>Yes*?</t>
+  </si>
+  <si>
+    <t>Answer displays twice. Seems like the source is a doc giving instructions on how Cidy should answer?</t>
+  </si>
+  <si>
+    <t>Answer: Yes, there is a Development Account (DA) checklist available for reviewing concept notes. The checklist is designed to assist DA Focal Points in reviewing each concept note before submission. It covers areas such as the use of the correct template, resource sufficiency, background context, target countries, project objectives, outcomes, outputs, UN system engagement, partnerships, and budget summary. The checklist ensures that all required sections are completed and that the concept note meets quality assurance standards prior to submission. This checklist is referenced as annex 2 in the 19th tranche guidelines and is specifically intended for internal quality review and pre-submission checks by implementing entities.
+Sources:
+​T19 Concept Note Review Checklist for DA Focal Points.docx​
+​T19 Concept Note Guidelines.docx​
+Confidence: Very High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer appears twice. </t>
+  </si>
+  <si>
+    <t>Answer: The responsibility for maintaining and updating the knowledge base used by Cidy lies with the Knowledge Control Center. This component tracks knowledge folders, source-use instructions, manager updates, route coverage, and YAML work needed to keep response topics aligned. Additionally, the governance and maintenance architecture includes an inventory generator to regenerate the knowledge inventory from the router and response YAMLs, a refresh workflow for synchronizing and updating files, and a structural test runner to check the inventory's support for expected flows. Human-in-the-loop processes are also in place, ensuring unresolved or low-confidence cases are escalated for human review rather than being treated as definitive answers. This approach ensures that Cidy's knowledge base remains accurate, current, and aligned with institutional requirements.
 Sources:
 ​Cidy - Architecture.docx​
 Confidence: Very High</t>
   </si>
   <si>
-    <t>Is this correct?</t>
-  </si>
-  <si>
-    <t>Did get asked multiple choice; DEBUG - Pass 2 result: Broad DA source (Pass 1 was blank)
-Query sent:
-Response:</t>
-  </si>
-  <si>
-    <t>Claude Found?</t>
-  </si>
-  <si>
-    <t>Happy path - DA project planning [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA project document [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA monitoring and reporting [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA budget eligibility [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA Section 35 signal [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA evaluation design [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA evaluation template [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA general start [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA latest tranche [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - DA checklist [DA]</t>
-  </si>
-  <si>
-    <t>Happy path - project evaluation evidence [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - evaluation recommendations [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - lessons learned [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - recurring evaluation findings [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - evaluation weaknesses [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - partnerships in evaluations [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - sustainability recommendations [Evaluation]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development CD Strategy [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development Steering Committee [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development TAG [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development general [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development annual progress report template [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development final report template [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development project document preparation [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development implementing partner agreement [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development grants due diligence [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development IPGC templates [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC budget and finance [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC governance [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC roles [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC programme design standards [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC evaluation criteria [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC reports [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - PDF / UNPDF [PDF]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy coverage [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy maintenance [About Cidy]</t>
-  </si>
-  <si>
-    <t>Clarification path - fund to DA [DA]</t>
-  </si>
-  <si>
-    <t>Clarification path - fund to RPTC [RPTC]</t>
-  </si>
-  <si>
-    <t>Clarification path - fund to PDF [PDF]</t>
-  </si>
-  <si>
-    <t>Clarification path - fund not sure [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain to DA [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain to Programme Development [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain to Evaluation Evidence [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain to About Cidy [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain to RPTC [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain typed DA [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain typed Development Account [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - domain typed UNPDF [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - artifact concept note [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - artifact evaluation report [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - artifact progress report [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - artifact management response [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - second attempt succeeds [Not Sure]</t>
-  </si>
-  <si>
-    <t>Clarification path - max attempts dead end [Not Sure]</t>
-  </si>
-  <si>
-    <t>Vague path - domain clarification [Not Sure]</t>
-  </si>
-  <si>
-    <t>Vague path - template clarification [Not Sure]</t>
-  </si>
-  <si>
-    <t>Vague path - report clarification [Not Sure]</t>
-  </si>
-  <si>
-    <t>Vague path - guidance clarification [Not Sure]</t>
-  </si>
-  <si>
-    <t>Vague path - project support clarification [Not Sure]</t>
-  </si>
-  <si>
-    <t>Out of scope - weather [OOS]</t>
-  </si>
-  <si>
-    <t>Out of scope - sports [OOS]</t>
-  </si>
-  <si>
-    <t>Out of scope - poem [OOS]</t>
-  </si>
-  <si>
-    <t>Out of scope - laptop help [OOS]</t>
-  </si>
-  <si>
-    <t>Out of scope - stock investment [OOS]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC activity proposal template [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC common reporting standards [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC IRA guidance [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC activity report template [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC planning and approval process [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC 2024 achievements [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC 2024 countries requests interventions [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC implementing entities [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC SIDS LDC LLDC support [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - RPTC future recommendations [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development Resident Coordinator mission notice [RPTC]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development UNSDCF alignment [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development UNCT membership [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development strategic priorities [PD]</t>
-  </si>
-  <si>
-    <t>Happy path - Programme Development service delivery model [PD]</t>
-  </si>
-  <si>
-    <t>Clarification path - Programme Development strategy from broad Cidy question [Not Sure]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy overview [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy comparison [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy user questions [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy prompt examples [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy routing flow [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy low confidence  [About Cidy]</t>
-  </si>
-  <si>
-    <t>Happy path - About Cidy architecture  [About Cidy]</t>
-  </si>
-  <si>
-    <t>Greeting path - English greeting only [Greeting]</t>
-  </si>
-  <si>
-    <t>Greeting path - Multilingual greeting only  [Greeting]</t>
-  </si>
-  <si>
-    <t>Greeting guard - greeting plus substantive question [Greeting]</t>
-  </si>
-  <si>
-    <t>Exit Cidy flow command - exact phrase [Exit Flow]</t>
-  </si>
-  <si>
-    <t>Exit Cidy flow command - Cindy typo [Exit Flow]</t>
-  </si>
-  <si>
-    <t>Return to Cidy rescue path  [Exit Flow]</t>
-  </si>
-  <si>
-    <t>Happy path - Country Data active projects by country [Country Data]</t>
-  </si>
-  <si>
-    <t>Regression - broad country work routes to Country Data [Country Data]</t>
-  </si>
-  <si>
-    <t>Happy path - Country Data proposal year list [Country Data]</t>
-  </si>
-  <si>
-    <t>Happy path - Country Data LDC activity count [Country Data]</t>
-  </si>
-  <si>
-    <t>Topic Area</t>
+    <t>Not really correct?</t>
+  </si>
+  <si>
+    <t>Unsure*</t>
   </si>
 </sst>
 </file>
@@ -1503,7 +1718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1514,30 +1729,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="19">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1551,21 +1748,6 @@
           <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1775,6 +1957,40 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1828,24 +2044,30 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TestCases" displayName="TestCases" ref="A1:N101" headerRowDxfId="18" dataDxfId="17" totalsRowDxfId="16">
-  <autoFilter ref="A1:N101" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:N101" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="DA"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{4A7C252B-E6AE-4BAB-8700-BD0D421264B4}" name="Topic Area" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="15"/>
+    <tableColumn id="14" xr3:uid="{4A7C252B-E6AE-4BAB-8700-BD0D421264B4}" name="Topic Area" dataDxfId="14">
       <calculatedColumnFormula>_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{592BE159-2946-4113-A670-6EF553577EF2}" name="General Notes" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{94470136-127C-457E-8281-70D3DB7C1FD4}" name="Claude Found?" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{592BE159-2946-4113-A670-6EF553577EF2}" name="General Notes" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{94470136-127C-457E-8281-70D3DB7C1FD4}" name="Claude Found?" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2170,27 +2392,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:N101"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="12" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="11.65" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.36328125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="32.26953125" style="4" customWidth="1"/>
-    <col min="4" max="5" width="32.26953125" style="3" customWidth="1"/>
-    <col min="6" max="9" width="12.90625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="9.7265625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.54296875" style="4" customWidth="1"/>
-    <col min="12" max="12" width="17.81640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="12.19921875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="32.265625" style="4" customWidth="1"/>
+    <col min="4" max="5" width="32.265625" style="3" customWidth="1"/>
+    <col min="6" max="9" width="12.9296875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="9.73046875" style="4" customWidth="1"/>
+    <col min="11" max="11" width="16.53125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="13" width="286" style="3" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" style="3" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="3"/>
+    <col min="14" max="14" width="15.46484375" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="8.73046875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -2199,25 +2421,25 @@
         <v>189</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>193</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>190</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>2</v>
@@ -2229,9 +2451,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="B2" s="3" t="str">
         <f t="shared" ref="B2:B33" si="0">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</f>
@@ -2240,24 +2462,24 @@
       <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>191</v>
+      <c r="D2" s="6" t="s">
+        <v>336</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>209</v>
+        <v>335</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G2" s="3"/>
       <c r="I2" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J2" s="5">
-        <v>46184</v>
+        <v>46194</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>198</v>
+        <v>337</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>6</v>
@@ -2266,9 +2488,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B3" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2277,21 +2499,24 @@
       <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>196</v>
+      <c r="D3" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>338</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>194</v>
+        <v>339</v>
       </c>
       <c r="G3" s="3"/>
       <c r="I3" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J3" s="5">
-        <v>46184</v>
+        <v>46194</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>198</v>
+        <v>337</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>6</v>
@@ -2300,9 +2525,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="B4" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2312,17 +2537,23 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>203</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G4" s="3"/>
+      <c r="I4" s="4" t="s">
+        <v>203</v>
+      </c>
       <c r="J4" s="5">
-        <v>46184</v>
+        <v>46194</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>198</v>
+        <v>337</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>6</v>
@@ -2331,9 +2562,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="B5" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2342,20 +2573,25 @@
       <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>201</v>
+      <c r="D5" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>342</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G5" s="3"/>
       <c r="I5" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J5" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K5" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L5" s="3" t="s">
         <v>6</v>
       </c>
@@ -2363,9 +2599,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="B6" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2374,18 +2610,25 @@
       <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E6" s="4"/>
+      <c r="D6" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>344</v>
+      </c>
       <c r="F6" s="3" t="s">
-        <v>200</v>
+        <v>339</v>
       </c>
       <c r="G6" s="3"/>
+      <c r="I6" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="J6" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K6" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L6" s="3" t="s">
         <v>6</v>
       </c>
@@ -2393,9 +2636,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="B7" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2404,20 +2647,25 @@
       <c r="C7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>202</v>
+      <c r="D7" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>346</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>194</v>
+        <v>339</v>
       </c>
       <c r="G7" s="3"/>
       <c r="I7" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J7" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K7" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L7" s="3" t="s">
         <v>6</v>
       </c>
@@ -2425,9 +2673,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="B8" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2436,20 +2684,25 @@
       <c r="C8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>202</v>
+      <c r="D8" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G8" s="3"/>
       <c r="I8" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J8" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K8" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L8" s="3" t="s">
         <v>6</v>
       </c>
@@ -2457,9 +2710,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="B9" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2471,17 +2724,22 @@
       <c r="D9" s="3" t="s">
         <v>203</v>
       </c>
+      <c r="E9" s="3" t="s">
+        <v>349</v>
+      </c>
       <c r="F9" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G9" s="3"/>
       <c r="I9" s="4" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="J9" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K9" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L9" s="3" t="s">
         <v>6</v>
       </c>
@@ -2489,9 +2747,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="B10" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2500,20 +2758,25 @@
       <c r="C10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>204</v>
+      <c r="D10" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>352</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>194</v>
+        <v>339</v>
       </c>
       <c r="G10" s="3"/>
       <c r="I10" s="4" t="s">
-        <v>200</v>
+        <v>351</v>
       </c>
       <c r="J10" s="5">
-        <v>46184</v>
-      </c>
-      <c r="K10" s="3"/>
+        <v>46194</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L10" s="3" t="s">
         <v>6</v>
       </c>
@@ -2521,9 +2784,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B11" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2532,18 +2795,25 @@
       <c r="C11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>205</v>
+      <c r="D11" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>354</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G11" s="3"/>
       <c r="I11" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+        <v>193</v>
+      </c>
+      <c r="J11" s="5">
+        <v>46194</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="L11" s="3" t="s">
         <v>6</v>
       </c>
@@ -2551,9 +2821,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B12" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2563,10 +2833,10 @@
         <v>26</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G12" s="3"/>
       <c r="J12" s="3"/>
@@ -2578,9 +2848,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="B13" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2600,9 +2870,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="B14" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2612,17 +2882,17 @@
         <v>30</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G14" s="3"/>
       <c r="I14" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J14" s="5">
         <v>46189</v>
@@ -2635,9 +2905,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="B15" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2647,17 +2917,17 @@
         <v>31</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G15" s="3"/>
       <c r="I15" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J15" s="5">
         <v>46189</v>
@@ -2670,9 +2940,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="B16" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2682,14 +2952,14 @@
         <v>33</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G16" s="3"/>
       <c r="I16" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J16" s="5">
         <v>46189</v>
@@ -2702,9 +2972,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="B17" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2714,23 +2984,23 @@
         <v>34</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G17" s="3"/>
       <c r="I17" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J17" s="5">
         <v>46189</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>6</v>
@@ -2739,9 +3009,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="B18" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2751,23 +3021,23 @@
         <v>35</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G18" s="3"/>
       <c r="I18" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J18" s="5">
         <v>46189</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>6</v>
@@ -2776,9 +3046,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="B19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2788,17 +3058,17 @@
         <v>36</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G19" s="3"/>
       <c r="I19" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J19" s="5">
         <v>46189</v>
@@ -2811,9 +3081,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="B20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2823,17 +3093,17 @@
         <v>37</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G20" s="3"/>
       <c r="I20" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J20" s="5">
         <v>46189</v>
@@ -2846,9 +3116,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="B21" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2858,17 +3128,17 @@
         <v>39</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G21" s="3"/>
       <c r="I21" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J21" s="5">
         <v>46189</v>
@@ -2881,9 +3151,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="B22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2893,14 +3163,14 @@
         <v>41</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G22" s="3"/>
       <c r="I22" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J22" s="5">
         <v>46189</v>
@@ -2913,9 +3183,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="B23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2925,17 +3195,17 @@
         <v>43</v>
       </c>
       <c r="D23" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="F23" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G23" s="3"/>
       <c r="I23" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J23" s="5">
         <v>46189</v>
@@ -2948,9 +3218,9 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="B24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2960,14 +3230,14 @@
         <v>45</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G24" s="3"/>
       <c r="I24" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J24" s="5">
         <v>46189</v>
@@ -2980,9 +3250,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="B25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2992,23 +3262,23 @@
         <v>47</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G25" s="3"/>
       <c r="I25" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J25" s="5">
         <v>46189</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>6</v>
@@ -3017,9 +3287,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="36" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="B26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3029,23 +3299,23 @@
         <v>48</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G26" s="3"/>
       <c r="I26" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J26" s="5">
         <v>46189</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>6</v>
@@ -3054,9 +3324,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="B27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3066,17 +3336,17 @@
         <v>49</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G27" s="3"/>
       <c r="I27" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J27" s="5">
         <v>46189</v>
@@ -3089,9 +3359,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="B28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3101,23 +3371,23 @@
         <v>51</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G28" s="3"/>
       <c r="I28" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J28" s="5">
         <v>46189</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>6</v>
@@ -3126,9 +3396,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="B29" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3138,23 +3408,23 @@
         <v>52</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G29" s="3"/>
       <c r="I29" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J29" s="5">
         <v>46189</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>6</v>
@@ -3163,9 +3433,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="B30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3175,23 +3445,23 @@
         <v>53</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G30" s="3"/>
       <c r="I30" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J30" s="5">
         <v>46189</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>6</v>
@@ -3200,9 +3470,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="B31" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3212,14 +3482,14 @@
         <v>55</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G31" s="3"/>
       <c r="I31" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J31" s="5">
         <v>46189</v>
@@ -3232,9 +3502,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="B32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3244,14 +3514,14 @@
         <v>56</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G32" s="3"/>
       <c r="I32" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J32" s="5">
         <v>46189</v>
@@ -3264,9 +3534,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="B33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3276,14 +3546,14 @@
         <v>57</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G33" s="3"/>
       <c r="I33" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J33" s="5">
         <v>46189</v>
@@ -3296,9 +3566,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="B34" s="3" t="str">
         <f t="shared" ref="B34:B65" si="1">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A34,"[",-1),"]")</f>
@@ -3308,14 +3578,14 @@
         <v>58</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G34" s="3"/>
       <c r="I34" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J34" s="5">
         <v>46189</v>
@@ -3328,9 +3598,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="B35" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3340,14 +3610,14 @@
         <v>59</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G35" s="3"/>
       <c r="I35" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J35" s="5">
         <v>46189</v>
@@ -3360,9 +3630,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="B36" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3372,14 +3642,14 @@
         <v>60</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G36" s="3"/>
       <c r="I36" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J36" s="5">
         <v>46189</v>
@@ -3392,9 +3662,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="B37" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3404,17 +3674,17 @@
         <v>62</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G37" s="3"/>
       <c r="I37" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J37" s="5">
         <v>46189</v>
@@ -3427,9 +3697,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="B38" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3439,14 +3709,14 @@
         <v>64</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G38" s="3"/>
       <c r="I38" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J38" s="5">
         <v>46189</v>
@@ -3459,9 +3729,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="B39" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3470,21 +3740,21 @@
       <c r="C39" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>243</v>
+      <c r="D39" s="6" t="s">
+        <v>355</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>244</v>
+        <v>356</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>194</v>
+        <v>339</v>
       </c>
       <c r="G39" s="3"/>
       <c r="I39" s="4" t="s">
-        <v>194</v>
+        <v>357</v>
       </c>
       <c r="J39" s="5">
-        <v>46189</v>
+        <v>46194</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3" t="s">
@@ -3494,9 +3764,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="B40" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3506,17 +3776,17 @@
         <v>67</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G40" s="3"/>
       <c r="I40" s="4" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="J40" s="5">
         <v>46189</v>
@@ -3529,9 +3799,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="B41" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3551,9 +3821,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="B42" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3573,9 +3843,9 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="B43" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3595,9 +3865,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="B44" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3617,9 +3887,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="B45" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3639,9 +3909,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="B46" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3661,9 +3931,9 @@
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="B47" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3683,9 +3953,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="B48" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3705,9 +3975,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="B49" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3727,9 +3997,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="B50" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3749,9 +4019,9 @@
         <v>95</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="B51" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3771,9 +4041,9 @@
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="B52" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3793,9 +4063,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="B53" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3815,9 +4085,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="B54" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3837,9 +4107,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="B55" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3859,9 +4129,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="B56" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3881,9 +4151,9 @@
         <v>113</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="B57" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3903,9 +4173,9 @@
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="B58" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3925,9 +4195,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="B59" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3947,9 +4217,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="B60" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3969,9 +4239,9 @@
         <v>120</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="B61" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3991,9 +4261,9 @@
         <v>122</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="B62" s="3" t="str">
         <f t="shared" si="1"/>
@@ -4013,9 +4283,9 @@
         <v>124</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="B63" s="3" t="str">
         <f t="shared" si="1"/>
@@ -4035,9 +4305,9 @@
         <v>126</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="B64" s="3" t="str">
         <f t="shared" si="1"/>
@@ -4057,9 +4327,9 @@
         <v>128</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="B65" s="3" t="str">
         <f t="shared" si="1"/>
@@ -4069,14 +4339,14 @@
         <v>129</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G65" s="3"/>
       <c r="H65" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
@@ -4087,9 +4357,9 @@
         <v>130</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="B66" s="3" t="str">
         <f t="shared" ref="B66:B97" si="2">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A66,"[",-1),"]")</f>
@@ -4109,9 +4379,9 @@
         <v>132</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="B67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4131,9 +4401,9 @@
         <v>132</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="B68" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4156,9 +4426,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="B69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4181,9 +4451,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="B70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4206,9 +4476,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="B71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4231,9 +4501,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="B72" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4256,9 +4526,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="B73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4281,9 +4551,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="B74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4306,9 +4576,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="B75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4331,9 +4601,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="B76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4356,9 +4626,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="B77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4381,9 +4651,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="B78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4406,9 +4676,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="B79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4431,9 +4701,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="B80" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4456,9 +4726,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="B81" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4481,9 +4751,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="B82" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4506,9 +4776,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="B83" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4531,9 +4801,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="B84" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4556,9 +4826,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="B85" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4581,9 +4851,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="B86" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4606,9 +4876,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" ht="34.9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="B87" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4631,9 +4901,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="B88" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4656,9 +4926,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="B89" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4681,9 +4951,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="B90" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4706,9 +4976,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="B91" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4731,9 +5001,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="B92" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4756,9 +5026,9 @@
         <v>168</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="3" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="B93" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4781,9 +5051,9 @@
         <v>168</v>
       </c>
     </row>
-    <row r="94" spans="1:14" ht="24" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:14" ht="23.25" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="3" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="B94" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4806,9 +5076,9 @@
         <v>168</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="3" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="B95" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4831,9 +5101,9 @@
         <v>174</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="B96" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4856,9 +5126,9 @@
         <v>174</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="3" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="B97" s="3" t="str">
         <f t="shared" si="2"/>
@@ -4881,12 +5151,12 @@
         <v>168</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="3" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="B98" s="3" t="str">
-        <f t="shared" ref="B98:B129" si="3">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A98,"[",-1),"]")</f>
+        <f t="shared" ref="B98:B101" si="3">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A98,"[",-1),"]")</f>
         <v>Country Data</v>
       </c>
       <c r="C98" s="4" t="s">
@@ -4906,9 +5176,9 @@
         <v>181</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="B99" s="3" t="str">
         <f t="shared" si="3"/>
@@ -4931,9 +5201,9 @@
         <v>184</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="B100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -4956,7 +5226,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:14" hidden="1" x14ac:dyDescent="0.35">
       <c r="B101" s="4" t="e">
         <f t="shared" si="3"/>
         <v>#VALUE!</v>
@@ -4980,10 +5250,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1:G1048576 I1:I1048576">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",F1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",F1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Updated DA broad search yaml and Jon excel
</commit_message>
<xml_diff>
--- a/documentation/Jons_Cidy_Intent_Test_Cases_90.xlsx
+++ b/documentation/Jons_Cidy_Intent_Test_Cases_90.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="500" documentId="13_ncr:1_{2B301336-FE44-41E3-9BB8-269871358495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6D28624-05C6-491C-B96C-EBDBB98883F8}"/>
   <bookViews>
-    <workbookView xWindow="315" yWindow="187" windowWidth="21083" windowHeight="12031" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35532" yWindow="540" windowWidth="21084" windowHeight="12036" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="388">
   <si>
     <t>Scenario</t>
   </si>
@@ -2137,7 +2137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2148,7 +2148,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2161,14 +2160,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2177,7 +2174,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="28">
     <dxf>
       <fill>
         <patternFill>
@@ -2233,74 +2230,6 @@
           <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -2455,7 +2384,61 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2596,28 +2579,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TestCases" displayName="TestCases" ref="A1:Q100" headerRowDxfId="29" dataDxfId="28" totalsRowDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TestCases" displayName="TestCases" ref="A1:Q100" headerRowDxfId="27" dataDxfId="26" totalsRowDxfId="25">
   <autoFilter ref="A1:Q100" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{4A7C252B-E6AE-4BAB-8700-BD0D421264B4}" name="Topic Area" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{4A7C252B-E6AE-4BAB-8700-BD0D421264B4}" name="Topic Area" dataDxfId="23">
       <calculatedColumnFormula>_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{592BE159-2946-4113-A670-6EF553577EF2}" name="General Notes" dataDxfId="22"/>
-    <tableColumn id="16" xr3:uid="{3626A57B-48DC-46B9-BCF8-BAFBC8E0C9ED}" name="Cidy's Route" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{D58229F1-875A-4B50-8450-24952B7178A5}" name="IsFallback?" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer 1 " dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{50FFC729-EC74-4E66-AF9B-3377B0EE5F51}" name="FoundAnswer 2" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{94470136-127C-457E-8281-70D3DB7C1FD4}" name="Claude Found?" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{592BE159-2946-4113-A670-6EF553577EF2}" name="General Notes" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{3626A57B-48DC-46B9-BCF8-BAFBC8E0C9ED}" name="Cidy's Route" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{D58229F1-875A-4B50-8450-24952B7178A5}" name="IsFallback?" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer 1 " dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{50FFC729-EC74-4E66-AF9B-3377B0EE5F51}" name="FoundAnswer 2" dataDxfId="16"/>
+    <tableColumn id="13" xr3:uid="{94470136-127C-457E-8281-70D3DB7C1FD4}" name="Claude Found?" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3022,7 +3005,7 @@
       <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>332</v>
       </c>
       <c r="E2" s="3" t="s">
@@ -3063,7 +3046,7 @@
       <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>336</v>
       </c>
       <c r="E3" s="3" t="s">
@@ -3139,7 +3122,7 @@
       <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="3" t="s">
         <v>337</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -3177,7 +3160,7 @@
       <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="3" t="s">
         <v>339</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -3215,7 +3198,7 @@
       <c r="C7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="3" t="s">
         <v>341</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -3291,7 +3274,7 @@
       <c r="C9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="3" t="s">
         <v>344</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -3329,7 +3312,7 @@
       <c r="C10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="3" t="s">
         <v>347</v>
       </c>
       <c r="E10" s="3" t="s">
@@ -4301,7 +4284,7 @@
       <c r="C38" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="3" t="s">
         <v>349</v>
       </c>
       <c r="E38" s="3" t="s">
@@ -5173,7 +5156,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="74" spans="1:17" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:17" ht="34.9" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>305</v>
       </c>
@@ -5875,10 +5858,10 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="H1:J1048576 L1:L1048576">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5908,484 +5891,484 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B2" s="11" t="str">
+      <c r="B2" s="10" t="str">
         <f t="shared" ref="B2:B10" si="0">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</f>
         <v>DA</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>371</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12" t="s">
+      <c r="J2" s="10"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="12">
         <v>46196</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="O2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="B3" s="16" t="str">
+      <c r="B3" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17" t="s">
+      <c r="J3" s="14"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="M3" s="21">
+      <c r="M3" s="18">
         <v>46196</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="25.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B4" s="11" t="str">
+      <c r="B4" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>372</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>374</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J4" s="11"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12" t="s">
+      <c r="J4" s="10"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="12">
         <v>46196</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="N4" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="P4" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="24.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B5" s="16" t="str">
+      <c r="B5" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J5" s="16"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17" t="s">
+      <c r="J5" s="14"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M5" s="21">
+      <c r="M5" s="18">
         <v>46196</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="P5" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12" t="s">
+      <c r="J6" s="10"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="12">
         <v>46196</v>
       </c>
-      <c r="N6" s="14" t="s">
+      <c r="N6" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="B7" s="16" t="str">
+      <c r="B7" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="14" t="s">
         <v>380</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17" t="s">
+      <c r="J7" s="14"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M7" s="21">
+      <c r="M7" s="18">
         <v>46196</v>
       </c>
-      <c r="N7" s="19" t="s">
+      <c r="N7" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O7" s="16" t="s">
+      <c r="O7" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P7" s="16" t="s">
+      <c r="P7" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B8" s="11" t="str">
+      <c r="B8" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="10" t="s">
         <v>381</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J8" s="11"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12" t="s">
+      <c r="J8" s="10"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="12">
         <v>46196</v>
       </c>
-      <c r="N8" s="14" t="s">
+      <c r="N8" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="B9" s="16" t="str">
+      <c r="B9" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17" t="s">
+      <c r="J9" s="14"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="18">
         <v>46196</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="N9" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O9" s="16" t="s">
+      <c r="O9" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P9" s="16" t="s">
+      <c r="P9" s="14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="11" t="str">
+      <c r="B10" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>386</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>385</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J10" s="11"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12" t="s">
+      <c r="J10" s="10"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="12">
         <v>46196</v>
       </c>
-      <c r="N10" s="14" t="s">
+      <c r="N10" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="P10" s="10" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1:J10 L1:L10">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6410,485 +6393,485 @@
     <col min="12" max="12" width="13.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B2" s="11" t="str">
+      <c r="B2" s="10" t="str">
         <f t="shared" ref="B2:B10" si="0">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</f>
         <v>DA</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12" t="s">
+      <c r="J2" s="10"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="12">
         <v>46196</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="O2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="B3" s="16" t="str">
+      <c r="B3" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17" t="s">
+      <c r="J3" s="14"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="M3" s="21">
+      <c r="M3" s="18">
         <v>46196</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="25.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B4" s="11" t="str">
+      <c r="B4" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J4" s="11"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12" t="s">
+      <c r="J4" s="10"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="12">
         <v>46196</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="N4" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="P4" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="24.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B5" s="16" t="str">
+      <c r="B5" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J5" s="16"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17" t="s">
+      <c r="J5" s="14"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M5" s="21">
+      <c r="M5" s="18">
         <v>46196</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="P5" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12" t="s">
+      <c r="J6" s="10"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="12">
         <v>46196</v>
       </c>
-      <c r="N6" s="14" t="s">
+      <c r="N6" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="B7" s="16" t="str">
+      <c r="B7" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17" t="s">
+      <c r="J7" s="14"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="M7" s="21">
+      <c r="M7" s="18">
         <v>46196</v>
       </c>
-      <c r="N7" s="19" t="s">
+      <c r="N7" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O7" s="16" t="s">
+      <c r="O7" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P7" s="16" t="s">
+      <c r="P7" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B8" s="11" t="str">
+      <c r="B8" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J8" s="11"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12" t="s">
+      <c r="J8" s="10"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="12">
         <v>46196</v>
       </c>
-      <c r="N8" s="14" t="s">
+      <c r="N8" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="B9" s="16" t="str">
+      <c r="B9" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17" t="s">
+      <c r="J9" s="14"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="18">
         <v>46196</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="N9" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O9" s="16" t="s">
+      <c r="O9" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P9" s="16" t="s">
+      <c r="P9" s="14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="11" t="str">
+      <c r="B10" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J10" s="11"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12" t="s">
+      <c r="J10" s="10"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="12">
         <v>46196</v>
       </c>
-      <c r="N10" s="14" t="s">
+      <c r="N10" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="P10" s="10" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1:J10 L1:L10">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6914,485 +6897,485 @@
     <col min="16" max="16" width="18.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B2" s="11" t="str">
+      <c r="B2" s="10" t="str">
         <f t="shared" ref="B2:B10" si="0">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A2,"[",-1),"]")</f>
         <v>DA</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12" t="s">
+      <c r="J2" s="10"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="12">
         <v>46196</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="O2" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="B3" s="16" t="str">
+      <c r="B3" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17" t="s">
+      <c r="J3" s="14"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="M3" s="21">
+      <c r="M3" s="18">
         <v>46196</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B4" s="11" t="str">
+      <c r="B4" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J4" s="11"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12" t="s">
+      <c r="J4" s="10"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="12">
         <v>46196</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="N4" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="P4" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B5" s="16" t="str">
+      <c r="B5" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J5" s="16"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17" t="s">
+      <c r="J5" s="14"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M5" s="21">
+      <c r="M5" s="18">
         <v>46196</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="P5" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12" t="s">
+      <c r="J6" s="10"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="12">
         <v>46196</v>
       </c>
-      <c r="N6" s="14" t="s">
+      <c r="N6" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="B7" s="16" t="str">
+      <c r="B7" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17" t="s">
+      <c r="J7" s="14"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M7" s="21">
+      <c r="M7" s="18">
         <v>46196</v>
       </c>
-      <c r="N7" s="19" t="s">
+      <c r="N7" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O7" s="16" t="s">
+      <c r="O7" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P7" s="16" t="s">
+      <c r="P7" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B8" s="11" t="str">
+      <c r="B8" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="J8" s="11"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12" t="s">
+      <c r="J8" s="10"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="12">
         <v>46196</v>
       </c>
-      <c r="N8" s="14" t="s">
+      <c r="N8" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="23.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="B9" s="16" t="str">
+      <c r="B9" s="14" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17" t="s">
+      <c r="J9" s="14"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="18">
         <v>46196</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="N9" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="O9" s="16" t="s">
+      <c r="O9" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="P9" s="16" t="s">
+      <c r="P9" s="14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="11" t="str">
+      <c r="B10" s="10" t="str">
         <f t="shared" si="0"/>
         <v>DA</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="J10" s="11"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12" t="s">
+      <c r="J10" s="10"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="12">
         <v>46196</v>
       </c>
-      <c r="N10" s="14" t="s">
+      <c r="N10" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="P10" s="10" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H1:J10 L1:L10">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",H1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>